<commit_message>
chore(campaign): fix human review packages + corpus provenance evidence
Rebuild xlsx/html with non-empty object_original/agency/source_row_hash,
E2E-aligned top20, real-corpus-provenance-gate, and honest package readiness.
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/CONFENGE-COMMERCIAL-READY-01/commercial-top20-human-review.xlsx
+++ b/artifacts/campaigns/CONFENGE-COMMERCIAL-READY-01/commercial-top20-human-review.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,45 +439,65 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>suggested_offer</t>
+          <t>alternative_offer</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>selected_offer_margin</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>supporting_signals</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>contradicting_signals</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>offer_scores</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>reviewer_1_label</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>reviewer_1_reason</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>reviewer_2_label</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>reviewer_2_reason</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>adjudicated_label</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>adjudicator</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>reviewed_at</t>
         </is>
@@ -486,500 +506,800 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>27254414000101</t>
+          <t>53640280000169</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FAK EMPREENDIMENTOS LTDA</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>9.5914</v>
+          <t>ENGENHARIA E COMERCIO RIGEL LTDA</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>licitacoes_propostas</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>["concurrent_portfolio", "agency_concentration"]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>["partial_mapping:renewal_risk", "partial_mapping:admin_load", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 1.54, "licitacoes_propostas_score": 4.4, "auditoria_orcamento_score": 0.0, "acompanhamento_contratual_score": 6.83, "gestao_documental_score": 3.208, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>95257945000108</t>
+          <t>47690102000140</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CONSTRUBRAS CONSTRUTORA LTDA</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>9.5276</v>
+          <t>FERMOPAR CONSTRUCOES LTDA</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>licitacoes_propostas</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>["concurrent_portfolio", "agency_concentration"]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>["partial_mapping:renewal_risk", "partial_mapping:admin_load", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 1.54, "licitacoes_propostas_score": 4.4, "auditoria_orcamento_score": 0.0, "acompanhamento_contratual_score": 6.23, "gestao_documental_score": 2.92, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13591585000103</t>
+          <t>33347913000138</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ARMANT SOLUCÕES EM CLIMATIZACAO LTDA</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>9.014099999999999</v>
+          <t>MIRANTE SERVICOS E LOCACOES LTDA</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>licitacoes_propostas</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.7703</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>["concurrent_portfolio", "agency_concentration", "contract_concentration"]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>["partial_mapping:renewal_risk", "partial_mapping:admin_load", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 1.54, "licitacoes_propostas_score": 4.4, "auditoria_orcamento_score": 0.05611159097579006, "acompanhamento_contratual_score": 5.170278977439475, "gestao_documental_score": 2.3440000000000003, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>15247296000117</t>
+          <t>34219868000107</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IBERICA CONSTRUÇÕES CIVIS E VIARIAS LTDA ME</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>8.9406</v>
+          <t>LGF CONSTRUTORA LTDA</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>licitacoes_propostas</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9514</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>["concurrent_portfolio", "agency_concentration", "contract_concentration"]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>["partial_mapping:renewal_risk", "partial_mapping:admin_load", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 1.2833333333333334, "licitacoes_propostas_score": 3.666666666666667, "auditoria_orcamento_score": 0.07522239954256969, "acompanhamento_contratual_score": 4.618055998856424, "gestao_documental_score": 2.0560000000000005, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>29084108000191</t>
+          <t>27254414000101</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AUTENTIKA CONSTRUÇÕES LTDA</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>8.655900000000001</v>
+          <t>FAK EMPREENDIMENTOS LTDA</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>licitacoes_propostas</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>4.7803</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>["concurrent_portfolio", "agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>["partial_mapping:admin_load", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 0.77, "licitacoes_propostas_score": 2.85, "auditoria_orcamento_score": 0.08011261159561157, "acompanhamento_contratual_score": 7.630281528989029, "gestao_documental_score": 1.4800000000000002, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>22798043000105</t>
+          <t>27743102000153</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KAENG INFRAESTRUTURA LTDA</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>8.5984</v>
+          <t>FJ CONSTRUTORA LTDA</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>licitacoes_propostas</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0.7633</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>["concurrent_portfolio", "agency_concentration"]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>["partial_mapping:renewal_risk", "partial_mapping:admin_load", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 1.2833333333333334, "licitacoes_propostas_score": 3.666666666666667, "auditoria_orcamento_score": 0.0, "acompanhamento_contratual_score": 4.43, "gestao_documental_score": 2.0560000000000005, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10558895000138</t>
+          <t>14190481000150</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NOROMIX CONCRETO S/A</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>8.4</v>
+          <t>MONTE CLARO CONSTRUCOES LTDA</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>licitacoes_propostas</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.8845</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>["concurrent_portfolio", "agency_concentration", "contract_concentration"]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>["partial_mapping:renewal_risk", "partial_mapping:admin_load", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 0.77, "licitacoes_propostas_score": 2.2, "auditoria_orcamento_score": 0.08160572940612071, "acompanhamento_contratual_score": 3.0845346295407885, "gestao_documental_score": 1.329454901057133, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>00472805000138</t>
+          <t>33220938000176</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TRACADO CONSTRUCOES E SERVICOS LTDA</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>8.4</v>
+          <t>CONSTROI EMPREITEIRA DE OBRAS E CONSTRUCOES LTDA</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>licitacoes_propostas</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>["concurrent_portfolio", "agency_concentration"]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>["partial_mapping:renewal_risk", "partial_mapping:admin_load", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 0.77, "licitacoes_propostas_score": 2.2, "auditoria_orcamento_score": 0.0, "acompanhamento_contratual_score": 3.23, "gestao_documental_score": 1.4800000000000002, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>00220982000127</t>
+          <t>28857380000102</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MATT CONSTRUTORA LTDA</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>8.4</v>
+          <t>TORRES E COSTA CONSTRUCAO LTDA</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>61608477000149</t>
+          <t>07814038000147</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DGB ENGENHARIA E CONSTRUCOES LTDA</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>8.4</v>
+          <t>EWERTON CHANANECO DE SOUZA LTDA</t>
+        </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06145928000140</t>
+          <t>40593578000113</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CONSTRUÇÃO CIVIL MG LTDA</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>8.4</v>
+          <t>E PEREIRA COSTA SERVICOS E COMERCIO</t>
+        </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>03094645000129</t>
+          <t>18245956000119</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>INFRASUL - INFRAESTRUTURA E EMPREENDIMENTOS LTDA</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>8.4</v>
+          <t>SOLIDA SERVICOS DE MAO DE OBRAS LTDA</t>
+        </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>21763372000140</t>
+          <t>39534812000152</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RIBEIRO E ANJOS EMPREENDIMENTOS E ENGENHARIA LTDA</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>8.4</v>
+          <t>CONSTRUTORA SANTA TEREZA LTDA</t>
+        </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10249046000100</t>
+          <t>00827454000130</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CONSTRUCOES SCHOROEDER LTDA</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>8.4</v>
+          <t>CERQUEIRA TORRES CONSTRUCOES TERRAPLENAGEM E PAVIMENTACAO LTDA</t>
+        </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>09223659000181</t>
+          <t>20594387000169</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>VIGA - PAVIMENTACAO E OBRAS LTDA.</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>8.4</v>
+          <t>ALTEON ENGENHARIA LTDA</t>
+        </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>26277170000101</t>
+          <t>00541146000144</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CONCRESUL ENGENHARIA LTDA</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>8.4</v>
+          <t>CONSTRUTORA PARAISO LTDA</t>
+        </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>43887548000108</t>
+          <t>15723058000130</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CONSTRUTORA SCHROEDER E SCHMIDT LTDA</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>8.4</v>
+          <t>JEFERSON SCHERMANN FERREIRA &amp; CIA LTDA</t>
+        </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>02740940000142</t>
+          <t>42786044000139</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>TERRA E TECNICA ENGENHARIA E EMPREENDIMENTOS LTDA</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>8.4</v>
+          <t>ENGEMATH CONSTRUCOES E SERVICOS LTDA</t>
+        </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>93336030000154</t>
+          <t>61917876000191</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ENPHASE PAVIMENTACOES LTDA</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>8.4</v>
+          <t>JLG PRESTACAO DE SERVICOS LTDA</t>
+        </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12535370000102</t>
+          <t>08756015000196</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>TERRABASE TERRAPLENAGEM LTDA</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>8.4</v>
+          <t>VIVA CONSTRUCOES E SERVICOS LTDA</t>
+        </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>acompanhamento_contratual</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>acompanhamento_admin</t>
+          <t>diagnostico_b2g</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>["agency_concentration", "contract_concentration", "near_expiry", "mapping:renewal_risk"]</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>["partial_mapping:market_entry", "nc:addendum_recurrence", "nc:adverse_event"]</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>{"diagnostico_b2g_score": 2.64, "licitacoes_propostas_score": 1.045, "auditoria_orcamento_score": 0.10800000000000001, "acompanhamento_contratual_score": 4.6, "gestao_documental_score": 0.6160000000000001, "inteligencia_pncp_score": 0.0}</t>
         </is>
       </c>
     </row>

</xml_diff>